<commit_message>
Add monthly vehicle report download
</commit_message>
<xml_diff>
--- a/VehicleLogBook_시설용_예시.xlsx
+++ b/VehicleLogBook_시설용_예시.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="58">
   <si>
     <t>항목명</t>
   </si>
@@ -108,6 +108,12 @@
     <t>기록ID</t>
   </si>
   <si>
+    <t>운행월</t>
+  </si>
+  <si>
+    <t>운행일자</t>
+  </si>
+  <si>
     <t>운행자</t>
   </si>
   <si>
@@ -139,6 +145,12 @@
   </si>
   <si>
     <t>예시-001</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
   </si>
   <si>
     <t>○○동 가정</t>
@@ -592,7 +604,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -645,7 +657,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -712,7 +724,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -808,36 +820,36 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>29</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>31</v>
-      </c>
       <c r="E1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" t="s">
         <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" t="s">
-        <v>33</v>
       </c>
       <c r="H1" t="s">
         <v>34</v>
@@ -857,51 +869,63 @@
       <c r="M1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2">
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2">
         <v>42351</v>
       </c>
-      <c r="H2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2">
+      <c r="J2" t="s">
+        <v>46</v>
+      </c>
+      <c r="K2">
         <v>42367</v>
       </c>
-      <c r="J2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2">
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2">
         <v>16</v>
       </c>
-      <c r="L2" t="s">
-        <v>44</v>
-      </c>
-      <c r="M2" t="s">
-        <v>42</v>
+      <c r="N2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -915,43 +939,43 @@
         <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>